<commit_message>
Publish US Quality Core 0.5.0 preview (Patient on US Core 8.0.1)
Rendered IG output from the uscore8_patient build. Download archives
(*.zip) are intentionally excluded per repo .gitignore; not needed for preview.

Generated with assistance from Claude Code
</commit_message>
<xml_diff>
--- a/docs/observations-summary.xlsx
+++ b/docs/observations-summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="23">
   <si>
     <t>Profile</t>
   </si>
@@ -45,6 +45,42 @@
   </si>
   <si>
     <t>Method</t>
+  </si>
+  <si>
+    <t>us-quality-core-observation-lab</t>
+  </si>
+  <si>
+    <t>US Quality Core Laboratory Result Observation</t>
+  </si>
+  <si>
+    <t>Observation Category Codes#laboratory</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/us/core/ValueSet/us-core-laboratory-test-codes (extensible)</t>
+  </si>
+  <si>
+    <t>dateTimeĵ, Periodĵ, Timingĵ, instantĵ</t>
+  </si>
+  <si>
+    <t>Quantityĵ, CodeableConceptĵ, stringĵ, booleanĵ, integerĵ, Rangeĵ, Ratioĵ, timeĵ, dateTimeĵ, Periodĵ</t>
+  </si>
+  <si>
+    <t>optional</t>
+  </si>
+  <si>
+    <t>us-quality-core-observation-screening-assessment</t>
+  </si>
+  <si>
+    <t>US Quality Core Observation Screening Assessment</t>
+  </si>
+  <si>
+    <t>Observation Category Codes#survey</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/us/core/ValueSet/us-core-survey-codes (preferred)</t>
   </si>
 </sst>
 </file>
@@ -166,10 +202,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyBorder="true" applyFill="true" applyFont="true">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyBorder="true" applyFill="true" applyAlignment="true" applyFont="true">
       <alignment vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment vertical="top" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -178,7 +214,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -216,6 +252,76 @@
         <v>10</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s" s="2">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="K2" t="s" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s" s="2">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="J3" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="K3" t="s" s="2">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>